<commit_message>
Update BOM_RheoboardV1.xlsx to reflect recent changes
- Modified the `BOM_RheoboardV1.xlsx` file to incorporate updated component information and ensure accuracy in sourcing. This change enhances the project's documentation and maintains the relevance of the BOM for users.
</commit_message>
<xml_diff>
--- a/RheoBoard_PCB/BOM/BOM_RheoboardV1.xlsx
+++ b/RheoBoard_PCB/BOM/BOM_RheoboardV1.xlsx
@@ -6,7 +6,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Bom từ kế toán" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,6 +68,12 @@
       <sz val="11"/>
       <u val="single"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <color rgb="FF0563C1"/>
+      <sz val="11"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Times New Roman"/>
@@ -143,7 +149,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -203,6 +209,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -804,8 +813,8 @@
     <col width="62.6640625" customWidth="1" style="4" min="5" max="5"/>
     <col width="12.5" customWidth="1" style="4" min="6" max="6"/>
     <col width="28.83203125" customWidth="1" style="4" min="7" max="7"/>
-    <col width="78" customWidth="1" style="4" min="8" max="10"/>
-    <col width="78" customWidth="1" style="4" min="11" max="16384"/>
+    <col width="78" customWidth="1" style="4" min="8" max="11"/>
+    <col width="78" customWidth="1" style="4" min="12" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -841,10 +850,14 @@
       </c>
       <c r="G1" s="26" t="inlineStr">
         <is>
-          <t>Mouser Link</t>
-        </is>
-      </c>
-      <c r="H1" s="10" t="n"/>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H1" s="26" t="inlineStr">
+        <is>
+          <t>Backup Link</t>
+        </is>
+      </c>
       <c r="I1" s="10" t="n"/>
       <c r="J1" s="10" t="n"/>
       <c r="K1" s="10" t="n"/>
@@ -1389,9 +1402,9 @@
           <t>C7393892</t>
         </is>
       </c>
-      <c r="G6" s="28" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Murata-Electronics/GRM188R61E106KA73D?qs=5aG0NVq1C4z8ebxPkQZf9A%3D%3D</t>
+      <c r="G6" s="31" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/Murata-Electronics/GRM188R61E106MA73D?qs=PoXZt%2B2CjACpktoD15Kv0Q%3D%3D</t>
         </is>
       </c>
       <c r="H6" s="10" t="n"/>
@@ -1499,9 +1512,9 @@
           <t>C20416420</t>
         </is>
       </c>
-      <c r="G7" s="28" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Samsung-Electro-Mechanics/CL21A226MAYNNNE?qs=xZ%2FP%2Ba9zWqY%2FVvCfXjMhqg%3D%3D</t>
+      <c r="G7" s="31" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/Murata-Electronics/GRM21BR61E226ME44K?qs=hNud%2FORuBR25jDsUehWlrQ%3D%3D</t>
         </is>
       </c>
       <c r="H7" s="10" t="n"/>
@@ -1609,9 +1622,9 @@
           <t>C2169079</t>
         </is>
       </c>
-      <c r="G8" s="27" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Vishay-Vitramon/VJ0603A180GXACW1BC?qs=fbqHpEqDHFJR%2BaVLLDw25A%3D%3D</t>
+      <c r="G8" s="31" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/YAGEO/CC0603JRNPO9BN180?qs=vTakOoo5QyKBbsg9i%2BJDzw%3D%3D</t>
         </is>
       </c>
       <c r="H8" s="10" t="n"/>
@@ -2202,7 +2215,7 @@
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>I2C_4</t>
+          <t>Qwiic (black)</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
@@ -2215,12 +2228,16 @@
           <t xml:space="preserve">C160404 </t>
         </is>
       </c>
-      <c r="G14" s="24" t="inlineStr">
+      <c r="G14" s="31" t="inlineStr">
+        <is>
+          <t>https://www.sparkfun.com/qwiic-jst-connector-smd-4-pin-horizontal.html</t>
+        </is>
+      </c>
+      <c r="H14" s="31" t="inlineStr">
         <is>
           <t>https://www.mouser.com/ProductDetail/JST-Commercial/SM04B-SRSS-TBLFSN?qs=cdbOS8ANM9B3FdyA6cNU2A%3D%3D</t>
         </is>
       </c>
-      <c r="H14" s="10" t="n"/>
       <c r="I14" s="10" t="n"/>
       <c r="J14" s="10" t="n"/>
       <c r="K14" s="10" t="n"/>
@@ -2402,7 +2419,7 @@
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>Khach Footprint:4.7uH_2A</t>
+          <t>4.7uH_2A</t>
         </is>
       </c>
       <c r="F16" s="19" t="inlineStr">
@@ -2520,9 +2537,9 @@
           <t>C25803</t>
         </is>
       </c>
-      <c r="G17" s="25" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Royalohm/0603WAF1003T5E?qs=e8oIoAS2J1SaaY9MznAX1w%3D%3D</t>
+      <c r="G17" s="31" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/YAGEO/RC0603FR-07100KL?qs=e1ok2LiJcmaihem8Va5%2Fsw%3D%3D</t>
         </is>
       </c>
       <c r="H17" s="10" t="n"/>
@@ -2630,9 +2647,9 @@
           <t>C4190</t>
         </is>
       </c>
-      <c r="G18" s="25" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Royalohm/0603WAF2201T5E?qs=e8oIoAS2J1Rz1NSs0bsVww%3D%3D</t>
+      <c r="G18" s="31" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/YAGEO/RC0603FR-072K2L?qs=diQw95jMAeOQmNpe2MM%2BPw%3D%3D</t>
         </is>
       </c>
       <c r="H18" s="10" t="n"/>
@@ -2850,9 +2867,9 @@
           <t>C22775</t>
         </is>
       </c>
-      <c r="G20" s="25" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Royalohm/0603WAF1000T5E?qs=e8oIoAS2J1QplezPhI1j8A%3D%3D</t>
+      <c r="G20" s="31" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/YAGEO/RC0603FR-07100RL?qs=NEN%2FsE%2FLsvPIwIWKCOS4%2FA%3D%3D</t>
         </is>
       </c>
       <c r="H20" s="10" t="n"/>
@@ -2960,9 +2977,9 @@
           <t>C25804</t>
         </is>
       </c>
-      <c r="G21" s="25" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Royalohm/0603WAF1002T5E?qs=e8oIoAS2J1TC2D0IjbSyGA%3D%3D</t>
+      <c r="G21" s="31" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/YAGEO/RC0603FR-0710KL?qs=grNVn54RoB%2B3GtjbJj3wJQ%3D%3D</t>
         </is>
       </c>
       <c r="H21" s="10" t="n"/>
@@ -3180,9 +3197,9 @@
           <t>C23138</t>
         </is>
       </c>
-      <c r="G23" s="25" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Royalohm/0603WAF3300T5E?qs=e8oIoAS2J1TtsqbFqPpAVg%3D%3D</t>
+      <c r="G23" s="31" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/YAGEO/RC0603FR-07330RL?qs=diQw95jMAeN1335dAOzMfg%3D%3D</t>
         </is>
       </c>
       <c r="H23" s="10" t="n"/>
@@ -3400,9 +3417,9 @@
           <t>C22984</t>
         </is>
       </c>
-      <c r="G25" s="25" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Royalohm/0603WAF3002T5E?qs=e8oIoAS2J1QKvIC%2FKcmyDw%3D%3D</t>
+      <c r="G25" s="31" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/YAGEO/RC0603FR-0730KL?qs=diQw95jMAeNFr44yr782FQ%3D%3D</t>
         </is>
       </c>
       <c r="H25" s="10" t="n"/>
@@ -3730,9 +3747,9 @@
           <t>C23079</t>
         </is>
       </c>
-      <c r="G28" s="27" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Royalohm/0603WAF5490T5E?qs=e8oIoAS2J1R4wIYcvgeFKg%3D%3D</t>
+      <c r="G28" s="31" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/YAGEO/RC0603FR-07549RL?qs=gt6vzsuosg3fZB4W1LlPKg%3D%3D</t>
         </is>
       </c>
       <c r="H28" s="10" t="n"/>
@@ -4165,7 +4182,11 @@
           <t>MPRLS0025PA00001A</t>
         </is>
       </c>
-      <c r="F32" s="19" t="n"/>
+      <c r="F32" s="19" t="inlineStr">
+        <is>
+          <t>C3257154</t>
+        </is>
+      </c>
       <c r="G32" s="27" t="inlineStr">
         <is>
           <t>https://www.mouser.com/ProductDetail/Honeywell/MPRLS0025PA00001A?qs=0lQeLiL1qyYP02EvUZH3dw%3D%3D</t>
@@ -4412,7 +4433,37 @@
       <c r="BG34" s="10" t="n"/>
     </row>
     <row r="35">
-      <c r="G35" s="10" t="n"/>
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>U4</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>TCA9534APWR</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>Khach Footprint:TCA9534APWR</t>
+        </is>
+      </c>
+      <c r="F35" s="19" t="inlineStr">
+        <is>
+          <t>C206010</t>
+        </is>
+      </c>
+      <c r="G35" s="30" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/Texas-Instruments/TCA9534APWR?qs=asCBFxFfL1RkU8XbvZBOXg%3D%3D</t>
+        </is>
+      </c>
       <c r="H35" s="10" t="n"/>
       <c r="I35" s="10" t="n"/>
       <c r="J35" s="10" t="n"/>
@@ -4467,7 +4518,37 @@
       <c r="BG35" s="10" t="n"/>
     </row>
     <row r="36">
-      <c r="G36" s="10" t="n"/>
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>U7</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>PCA9685PW</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>Khach Footprint:PCA9685</t>
+        </is>
+      </c>
+      <c r="F36" s="19" t="inlineStr">
+        <is>
+          <t>C2678753</t>
+        </is>
+      </c>
+      <c r="G36" s="30" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/NXP-Semiconductors/PCA9685PW118?qs=6YAT8rHPFU%2BtfwwKq4nwEQ%3D%3D</t>
+        </is>
+      </c>
       <c r="H36" s="10" t="n"/>
       <c r="I36" s="10" t="n"/>
       <c r="J36" s="10" t="n"/>
@@ -4522,7 +4603,37 @@
       <c r="BG36" s="10" t="n"/>
     </row>
     <row r="37">
-      <c r="G37" s="10" t="n"/>
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>Q3,Q4,Q8,Q10</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>AO3400A</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>Khach Footprint:AO3400A</t>
+        </is>
+      </c>
+      <c r="F37" s="19" t="inlineStr">
+        <is>
+          <t>C20917</t>
+        </is>
+      </c>
+      <c r="G37" s="31" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/alpha-omega-semiconductor-inc/AO3400A/1856105</t>
+        </is>
+      </c>
       <c r="H37" s="10" t="n"/>
       <c r="I37" s="10" t="n"/>
       <c r="J37" s="10" t="n"/>
@@ -4577,7 +4688,37 @@
       <c r="BG37" s="10" t="n"/>
     </row>
     <row r="38">
-      <c r="G38" s="10" t="n"/>
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>C32,C34,C43,C45</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>100uF/16V</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>Capacitor_SMD:CP_Elec_6.3x5.4_Nichicon</t>
+        </is>
+      </c>
+      <c r="F38" s="19" t="inlineStr">
+        <is>
+          <t>C128532</t>
+        </is>
+      </c>
+      <c r="G38" s="31" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/Panasonic-Industry/EEE-FK1C101P?qs=qE6bgDGEOCuSC5c%2BLSbo8Q%3D%3D</t>
+        </is>
+      </c>
       <c r="H38" s="10" t="n"/>
       <c r="I38" s="10" t="n"/>
       <c r="J38" s="10" t="n"/>
@@ -13611,30 +13752,35 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId34"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId39"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>